<commit_message>
Finalizing Official Comedy List
</commit_message>
<xml_diff>
--- a/Comedy_Whitelist.xlsx
+++ b/Comedy_Whitelist.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bigba\aa Personal Projects\Letterboxd-List-Scraping\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A363068-4145-4327-BCF3-1D0C373531E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6FA3610-C400-42EF-B278-8D88400C211F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="266">
   <si>
     <t>Title</t>
   </si>
@@ -28,22 +28,34 @@
     <t>Year</t>
   </si>
   <si>
+    <t>tmdbId</t>
+  </si>
+  <si>
     <t>Link</t>
   </si>
   <si>
     <t>James Acaster: Cold Lasagne Hate Myself 1999</t>
   </si>
   <si>
+    <t>2020</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/james-acaster-cold-lasagne-hate-myself-1999/</t>
   </si>
   <si>
     <t>Daniel Sloss: X</t>
   </si>
   <si>
+    <t>2019</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/daniel-sloss-x/</t>
   </si>
   <si>
-    <t>Dave Chappelle: Killinâ€™ Them Softly</t>
+    <t>Dave Chappelle: Killinâ€TM Them Softly</t>
+  </si>
+  <si>
+    <t>2000</t>
   </si>
   <si>
     <t>https://letterboxd.com/film/dave-chappelle-killin-them-softly/</t>
@@ -52,36 +64,54 @@
     <t>John Mulaney: New in Town</t>
   </si>
   <si>
+    <t>2012</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/john-mulaney-new-in-town/</t>
   </si>
   <si>
     <t>CMYLMZ</t>
   </si>
   <si>
+    <t>2008</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/cmylmz/</t>
   </si>
   <si>
     <t>Color Theories by Julio Torres. A Guide to Seeing the World</t>
   </si>
   <si>
+    <t>2026</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/color-theories-by-julio-torres-a-guide-to/</t>
   </si>
   <si>
     <t>Jerrod Carmichael: Rothaniel</t>
   </si>
   <si>
+    <t>2022</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/jerrod-carmichael-rothaniel/</t>
   </si>
   <si>
     <t>Bo Burnham: Make Happy</t>
   </si>
   <si>
+    <t>2016</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/bo-burnham-make-happy/</t>
   </si>
   <si>
     <t>John Mulaney: Kid Gorgeous at Radio City</t>
   </si>
   <si>
+    <t>2018</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/john-mulaney-kid-gorgeous-at-radio-city/</t>
   </si>
   <si>
@@ -94,25 +124,40 @@
     <t>Stand Up Solutions</t>
   </si>
   <si>
+    <t>2024</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/stand-up-solutions/</t>
   </si>
   <si>
+    <t>08:46:00</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/8-46-2020/</t>
   </si>
   <si>
     <t>John Mulaney: The Comeback Kid</t>
   </si>
   <si>
+    <t>2015</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/john-mulaney-the-comeback-kid/</t>
   </si>
   <si>
-    <t>George Carlin: Jamminâ€™ in New York</t>
+    <t>George Carlin: Jamminâ€TM in New York</t>
+  </si>
+  <si>
+    <t>1992</t>
   </si>
   <si>
     <t>https://letterboxd.com/film/george-carlin-jammin-in-new-york/</t>
   </si>
   <si>
-    <t>Dave Chappelle: For What Itâ€™s Worth</t>
+    <t>Dave Chappelle: For What Itâ€TMs Worth</t>
+  </si>
+  <si>
+    <t>2004</t>
   </si>
   <si>
     <t>https://letterboxd.com/film/dave-chappelle-for-what-its-worth/</t>
@@ -121,22 +166,31 @@
     <t>Eddie Izzard: Dress to Kill</t>
   </si>
   <si>
+    <t>1999</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/eddie-izzard-dress-to-kill/</t>
   </si>
   <si>
     <t>Norm Macdonald: Me Doing Standup</t>
   </si>
   <si>
+    <t>2011</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/norm-macdonald-me-doing-standup/</t>
   </si>
   <si>
     <t>Joe Pera: Slow &amp; Steady</t>
   </si>
   <si>
+    <t>2023</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/joe-pera-slow-steady/</t>
   </si>
   <si>
-    <t>Patrice Oâ€™Neal: Elephant in the Room</t>
+    <t>Patrice Oâ€TMNeal: Elephant in the Room</t>
   </si>
   <si>
     <t>https://letterboxd.com/film/patrice-oneal-elephant-in-the-room/</t>
@@ -145,12 +199,18 @@
     <t>George Carlin: Back in Town</t>
   </si>
   <si>
+    <t>1996</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/george-carlin-back-in-town/</t>
   </si>
   <si>
     <t>One Night Stand: Flight of the Conchords</t>
   </si>
   <si>
+    <t>2005</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/one-night-stand-flight-of-the-conchords/</t>
   </si>
   <si>
@@ -169,18 +229,27 @@
     <t>Hasan Minhaj: Homecoming King</t>
   </si>
   <si>
+    <t>2017</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/hasan-minhaj-homecoming-king/</t>
   </si>
   <si>
     <t>Bo Burnham: What.</t>
   </si>
   <si>
+    <t>2013</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/bo-burnham-what/</t>
   </si>
   <si>
     <t>Richard Pryor: Live in Concert</t>
   </si>
   <si>
+    <t>1979</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/richard-pryor-live-in-concert/</t>
   </si>
   <si>
@@ -193,6 +262,9 @@
     <t>Bill Hicks: Relentless</t>
   </si>
   <si>
+    <t>2006</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/bill-hicks-relentless/</t>
   </si>
   <si>
@@ -205,10 +277,13 @@
     <t>Shane Gillis: Live in Austin</t>
   </si>
   <si>
+    <t>2021</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/shane-gillis-live-in-austin/</t>
   </si>
   <si>
-    <t>George Carlin: Itâ€™s Bad for Ya!</t>
+    <t>George Carlin: Itâ€TMs Bad for Ya!</t>
   </si>
   <si>
     <t>https://letterboxd.com/film/george-carlin-its-bad-for-ya/</t>
@@ -217,6 +292,9 @@
     <t>Louis C.K.: Hilarious</t>
   </si>
   <si>
+    <t>2010</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/louis-ck-hilarious/</t>
   </si>
   <si>
@@ -247,12 +325,18 @@
     <t>Bill Hicks: Revelations</t>
   </si>
   <si>
+    <t>1993</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/bill-hicks-revelations/</t>
   </si>
   <si>
     <t>Louis C.K.: Shameless</t>
   </si>
   <si>
+    <t>2007</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/louis-ck-shameless/</t>
   </si>
   <si>
@@ -277,6 +361,9 @@
     <t>Gianmarco Soresi: Thief of Joy</t>
   </si>
   <si>
+    <t>2025</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/gianmarco-soresi-thief-of-joy/</t>
   </si>
   <si>
@@ -301,12 +388,18 @@
     <t>Robin Williams: Live on Broadway</t>
   </si>
   <si>
+    <t>2002</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/robin-williams-live-on-broadway/</t>
   </si>
   <si>
     <t>George Carlin: Complaints &amp; Grievances</t>
   </si>
   <si>
+    <t>2001</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/george-carlin-complaints-grievances/</t>
   </si>
   <si>
@@ -316,13 +409,13 @@
     <t>https://letterboxd.com/film/alex-edelman-just-for-us/</t>
   </si>
   <si>
-    <t>Mike Birbiglia: My Girlfriendâ€™s Boyfriend</t>
+    <t>Mike Birbiglia: My Girlfriendâ€TMs Boyfriend</t>
   </si>
   <si>
     <t>https://letterboxd.com/film/mike-birbiglia-my-girlfriends-boyfriend/</t>
   </si>
   <si>
-    <t>Daniel Howell: WEâ€™RE ALL DOOMED!</t>
+    <t>Daniel Howell: WEâ€TMRE ALL DOOMED!</t>
   </si>
   <si>
     <t>https://letterboxd.com/film/daniel-howell-were-all-doomed/</t>
@@ -370,7 +463,10 @@
     <t>https://letterboxd.com/film/dave-chappelle-equanimity/</t>
   </si>
   <si>
-    <t>George Carlin: Doinâ€™ It Again</t>
+    <t>George Carlin: Doinâ€TM It Again</t>
+  </si>
+  <si>
+    <t>1990</t>
   </si>
   <si>
     <t>https://letterboxd.com/film/george-carlin-doin-it-again/</t>
@@ -397,6 +493,9 @@
     <t>Bill Hicks: Sane Man</t>
   </si>
   <si>
+    <t>1989</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/bill-hicks-sane-man/</t>
   </si>
   <si>
@@ -421,6 +520,9 @@
     <t>An Evening with Robin Williams</t>
   </si>
   <si>
+    <t>1983</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/an-evening-with-robin-williams/</t>
   </si>
   <si>
@@ -445,6 +547,9 @@
     <t>Richard Pryor: Live on the Sunset Strip</t>
   </si>
   <si>
+    <t>1982</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/richard-pryor-live-on-the-sunset-strip/</t>
   </si>
   <si>
@@ -454,14 +559,272 @@
     <t>https://letterboxd.com/film/demi-adejuyigbe-is-going-to-do-one-1-backflip/</t>
   </si>
   <si>
-    <t>tmdbId</t>
+    <t>Jim Jefferies: Alcoholocaust</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/jim-jefferies-alcoholocaust/</t>
+  </si>
+  <si>
+    <t>Shane Gillis: Beautiful Dogs</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/shane-gillis-beautiful-dogs/</t>
+  </si>
+  <si>
+    <t>Kate Berlant: Cinnamon in the Wind</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/kate-berlant-cinnamon-in-the-wind/</t>
+  </si>
+  <si>
+    <t>Mike Birbiglia: The New One</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/mike-birbiglia-the-new-one/</t>
+  </si>
+  <si>
+    <t>Bill Burr: Iâ€TMm Sorry You Feel That Way</t>
+  </si>
+  <si>
+    <t>2014</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/bill-burr-im-sorry-you-feel-that-way/</t>
+  </si>
+  <si>
+    <t>Mark Normand: Out To Lunch</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/mark-normand-out-to-lunch/</t>
+  </si>
+  <si>
+    <t>Eddie Izzard: Glorious</t>
+  </si>
+  <si>
+    <t>1997</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/eddie-izzard-glorious/</t>
+  </si>
+  <si>
+    <t>Bill Burr: You People Are All The Same</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/bill-burr-you-people-are-all-the-same/</t>
+  </si>
+  <si>
+    <t>Robin Williams: An Evening at the Met</t>
+  </si>
+  <si>
+    <t>1986</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/robin-williams-an-evening-at-the-met/</t>
+  </si>
+  <si>
+    <t>This Filthy World</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/this-filthy-world/</t>
+  </si>
+  <si>
+    <t>Hasan Minhaj: The Kingâ€TMs Jester</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/hasan-minhaj-the-kings-jester/</t>
+  </si>
+  <si>
+    <t>Dave Chappelle: The Bird Revelation</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/dave-chappelle-the-bird-revelation/</t>
+  </si>
+  <si>
+    <t>John Mulaney: Baby J</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/john-mulaney-baby-j/</t>
+  </si>
+  <si>
+    <t>John Early: Now More Than Ever</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/john-early-now-more-than-ever/</t>
+  </si>
+  <si>
+    <t>Sincerely Louis C.K.</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/sincerely-louis-ck/</t>
+  </si>
+  <si>
+    <t>Chris Rock: Never Scared</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/chris-rock-never-scared/</t>
+  </si>
+  <si>
+    <t>Louis C.K.: One Night Stand</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/louis-ck-one-night-stand/</t>
+  </si>
+  <si>
+    <t>Dave Chappelle: The Age of Spin</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/dave-chappelle-the-age-of-spin/</t>
+  </si>
+  <si>
+    <t>Zakir Khan: Tathastu</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/zakir-khan-tathastu/</t>
+  </si>
+  <si>
+    <t>Neal Brennan: 3 Mics</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/neal-brennan-3-mics/</t>
+  </si>
+  <si>
+    <t>Louis C.K. at The Dolby</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/louis-ck-at-the-dolby/</t>
+  </si>
+  <si>
+    <t>My Favorite Shapes by Julio Torres</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/my-favorite-shapes-by-julio-torres/</t>
+  </si>
+  <si>
+    <t>Sam Morril: I Got This</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/sam-morril-i-got-this/</t>
+  </si>
+  <si>
+    <t>Caleb Hearon: Model Comedian</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/caleb-hearon-model-comedian/</t>
+  </si>
+  <si>
+    <t>George Carlin: What Am I Doing in New Jersey?</t>
+  </si>
+  <si>
+    <t>1988</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/george-carlin-what-am-i-doing-in-new-jersey/</t>
+  </si>
+  <si>
+    <t>Sheng Wang: Sweet and Juicy</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/sheng-wang-sweet-and-juicy/</t>
+  </si>
+  <si>
+    <t>Fabrice Ã‰bouÃ© - Adieu Hier</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/fabrice-eboue-adieu-hier/</t>
+  </si>
+  <si>
+    <t>Jim Carrey: Unnatural Act</t>
+  </si>
+  <si>
+    <t>1991</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/jim-carrey-unnatural-act/</t>
+  </si>
+  <si>
+    <t>Nick Mullen: The Year of the Dragon</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/nick-mullen-the-year-of-the-dragon/</t>
+  </si>
+  <si>
+    <t>Stewart Lee: Snowflake</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/stewart-lee-snowflake/</t>
+  </si>
+  <si>
+    <t>Hank Green: Pissing Out Cancer</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/hank-green-pissing-out-cancer/</t>
+  </si>
+  <si>
+    <t>Ricky Gervais: Out of England 2</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/ricky-gervais-out-of-england-2/</t>
+  </si>
+  <si>
+    <t>Bo Burnham: Words, Words, Words</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/bo-burnham-words-words-words/</t>
+  </si>
+  <si>
+    <t>Robin Williams: Weapons of Self Destruction</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/robin-williams-weapons-of-self-destruction/</t>
+  </si>
+  <si>
+    <t>Hannibal Buress: Animal Furnace</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/hannibal-buress-animal-furnace/</t>
+  </si>
+  <si>
+    <t>Norm Macdonald: Hitlerâ€™s Dog, Gossip &amp; Trickery</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/norm-macdonald-hitlers-dog-gossip-trickery/</t>
+  </si>
+  <si>
+    <t>Taylor Tomlinson: Look at You</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/taylor-tomlinson-look-at-you/</t>
+  </si>
+  <si>
+    <t>Judah Friedlander: America Is the Greatest Country in the United States</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/judah-friedlander-america-is-the-greatest-country-in-the-united-states/</t>
+  </si>
+  <si>
+    <t>Ricky Gervais Live: Animals</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/ricky-gervais-live-animals/</t>
+  </si>
+  <si>
+    <t>Mike Birbiglia: Thank God for Jokes</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/mike-birbiglia-thank-god-for-jokes/</t>
+  </si>
+  <si>
+    <t>Donald Glover: Weirdo</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/donald-glover-weirdo/</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -473,6 +836,14 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -507,17 +878,19 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -818,7 +1191,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D72"/>
+  <dimension ref="A1:D113"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
@@ -829,1007 +1202,1585 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>144</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2">
-        <v>2020</v>
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
       </c>
       <c r="C2">
         <v>763274</v>
       </c>
       <c r="D2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3">
-        <v>2019</v>
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
       </c>
       <c r="C3">
         <v>637573</v>
       </c>
       <c r="D3" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4">
-        <v>2000</v>
+        <v>10</v>
+      </c>
+      <c r="B4" t="s">
+        <v>11</v>
       </c>
       <c r="C4">
         <v>16275</v>
       </c>
       <c r="D4" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5">
-        <v>2012</v>
+        <v>13</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
       </c>
       <c r="C5">
         <v>86705</v>
       </c>
       <c r="D5" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6">
-        <v>2008</v>
+        <v>16</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
       </c>
       <c r="C6">
         <v>80981</v>
       </c>
       <c r="D6" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7">
-        <v>2026</v>
+        <v>19</v>
+      </c>
+      <c r="B7" t="s">
+        <v>20</v>
       </c>
       <c r="C7">
         <v>1573688</v>
       </c>
       <c r="D7" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8">
-        <v>2022</v>
+        <v>22</v>
+      </c>
+      <c r="B8" t="s">
+        <v>23</v>
       </c>
       <c r="C8">
         <v>952326</v>
       </c>
       <c r="D8" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>17</v>
-      </c>
-      <c r="B9">
-        <v>2016</v>
+        <v>25</v>
+      </c>
+      <c r="B9" t="s">
+        <v>26</v>
       </c>
       <c r="C9">
         <v>400608</v>
       </c>
       <c r="D9" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>19</v>
-      </c>
-      <c r="B10">
-        <v>2018</v>
+        <v>28</v>
+      </c>
+      <c r="B10" t="s">
+        <v>29</v>
       </c>
       <c r="C10">
         <v>520594</v>
       </c>
       <c r="D10" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>21</v>
-      </c>
-      <c r="B11">
-        <v>2018</v>
+        <v>31</v>
+      </c>
+      <c r="B11" t="s">
+        <v>29</v>
       </c>
       <c r="C11">
         <v>529531</v>
       </c>
       <c r="D11" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>23</v>
-      </c>
-      <c r="B12">
-        <v>2024</v>
+        <v>33</v>
+      </c>
+      <c r="B12" t="s">
+        <v>34</v>
       </c>
       <c r="C12">
         <v>1290099</v>
       </c>
       <c r="D12" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" s="2">
-        <v>0.36527777777777776</v>
-      </c>
-      <c r="B13">
-        <v>2020</v>
+      <c r="A13" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" t="s">
+        <v>5</v>
       </c>
       <c r="C13">
         <v>714842</v>
       </c>
       <c r="D13" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14">
-        <v>2015</v>
+        <v>38</v>
+      </c>
+      <c r="B14" t="s">
+        <v>39</v>
       </c>
       <c r="C14">
         <v>367735</v>
       </c>
       <c r="D14" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>28</v>
-      </c>
-      <c r="B15">
-        <v>1992</v>
+        <v>41</v>
+      </c>
+      <c r="B15" t="s">
+        <v>42</v>
       </c>
       <c r="C15">
         <v>25161</v>
       </c>
       <c r="D15" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>30</v>
-      </c>
-      <c r="B16">
-        <v>2004</v>
+        <v>44</v>
+      </c>
+      <c r="B16" t="s">
+        <v>45</v>
       </c>
       <c r="C16">
         <v>20147</v>
       </c>
       <c r="D16" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>32</v>
-      </c>
-      <c r="B17">
-        <v>1999</v>
+        <v>47</v>
+      </c>
+      <c r="B17" t="s">
+        <v>48</v>
       </c>
       <c r="C17">
         <v>13589</v>
       </c>
       <c r="D17" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>34</v>
-      </c>
-      <c r="B18">
-        <v>2011</v>
+        <v>50</v>
+      </c>
+      <c r="B18" t="s">
+        <v>51</v>
       </c>
       <c r="C18">
         <v>60233</v>
       </c>
       <c r="D18" t="s">
-        <v>35</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>36</v>
-      </c>
-      <c r="B19">
-        <v>2023</v>
+        <v>53</v>
+      </c>
+      <c r="B19" t="s">
+        <v>54</v>
       </c>
       <c r="C19">
         <v>1179932</v>
       </c>
       <c r="D19" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>38</v>
-      </c>
-      <c r="B20">
-        <v>2011</v>
+        <v>56</v>
+      </c>
+      <c r="B20" t="s">
+        <v>51</v>
       </c>
       <c r="C20">
         <v>57469</v>
       </c>
       <c r="D20" t="s">
-        <v>39</v>
+        <v>57</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>40</v>
-      </c>
-      <c r="B21">
-        <v>1996</v>
+        <v>58</v>
+      </c>
+      <c r="B21" t="s">
+        <v>59</v>
       </c>
       <c r="C21">
         <v>34509</v>
       </c>
       <c r="D21" t="s">
-        <v>41</v>
+        <v>60</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>42</v>
-      </c>
-      <c r="B22">
-        <v>2005</v>
+        <v>61</v>
+      </c>
+      <c r="B22" t="s">
+        <v>62</v>
       </c>
       <c r="C22">
         <v>147502</v>
       </c>
       <c r="D22" t="s">
-        <v>43</v>
+        <v>63</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>44</v>
-      </c>
-      <c r="B23">
-        <v>1992</v>
+        <v>64</v>
+      </c>
+      <c r="B23" t="s">
+        <v>42</v>
       </c>
       <c r="C23">
         <v>18458</v>
       </c>
       <c r="D23" t="s">
-        <v>45</v>
+        <v>65</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>46</v>
-      </c>
-      <c r="B24">
-        <v>2018</v>
+        <v>66</v>
+      </c>
+      <c r="B24" t="s">
+        <v>29</v>
       </c>
       <c r="C24">
         <v>550416</v>
       </c>
       <c r="D24" t="s">
-        <v>47</v>
+        <v>67</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>48</v>
-      </c>
-      <c r="B25">
-        <v>2017</v>
+        <v>68</v>
+      </c>
+      <c r="B25" t="s">
+        <v>69</v>
       </c>
       <c r="C25">
         <v>458310</v>
       </c>
       <c r="D25" t="s">
-        <v>49</v>
+        <v>70</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>50</v>
-      </c>
-      <c r="B26">
-        <v>2013</v>
+        <v>71</v>
+      </c>
+      <c r="B26" t="s">
+        <v>72</v>
       </c>
       <c r="C26">
         <v>244001</v>
       </c>
       <c r="D26" t="s">
-        <v>51</v>
+        <v>73</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>52</v>
-      </c>
-      <c r="B27">
-        <v>1979</v>
+        <v>74</v>
+      </c>
+      <c r="B27" t="s">
+        <v>75</v>
       </c>
       <c r="C27">
         <v>22975</v>
       </c>
       <c r="D27" t="s">
-        <v>53</v>
+        <v>76</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>54</v>
-      </c>
-      <c r="B28">
-        <v>1999</v>
+        <v>77</v>
+      </c>
+      <c r="B28" t="s">
+        <v>48</v>
       </c>
       <c r="C28">
         <v>34513</v>
       </c>
       <c r="D28" t="s">
-        <v>55</v>
+        <v>78</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>56</v>
-      </c>
-      <c r="B29">
-        <v>2006</v>
+        <v>79</v>
+      </c>
+      <c r="B29" t="s">
+        <v>80</v>
       </c>
       <c r="C29">
         <v>34505</v>
       </c>
       <c r="D29" t="s">
-        <v>57</v>
+        <v>81</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>58</v>
-      </c>
-      <c r="B30">
-        <v>2008</v>
+        <v>82</v>
+      </c>
+      <c r="B30" t="s">
+        <v>17</v>
       </c>
       <c r="C30">
         <v>30969</v>
       </c>
       <c r="D30" t="s">
-        <v>59</v>
+        <v>83</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>60</v>
-      </c>
-      <c r="B31">
-        <v>2021</v>
+        <v>84</v>
+      </c>
+      <c r="B31" t="s">
+        <v>85</v>
       </c>
       <c r="C31">
         <v>872209</v>
       </c>
       <c r="D31" t="s">
-        <v>61</v>
+        <v>86</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>62</v>
-      </c>
-      <c r="B32">
-        <v>2008</v>
+        <v>87</v>
+      </c>
+      <c r="B32" t="s">
+        <v>17</v>
       </c>
       <c r="C32">
         <v>13643</v>
       </c>
       <c r="D32" t="s">
-        <v>63</v>
+        <v>88</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>64</v>
-      </c>
-      <c r="B33">
-        <v>2010</v>
+        <v>89</v>
+      </c>
+      <c r="B33" t="s">
+        <v>90</v>
       </c>
       <c r="C33">
         <v>45523</v>
       </c>
       <c r="D33" t="s">
-        <v>65</v>
+        <v>91</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>66</v>
-      </c>
-      <c r="B34">
-        <v>2024</v>
+        <v>92</v>
+      </c>
+      <c r="B34" t="s">
+        <v>34</v>
       </c>
       <c r="C34">
         <v>1214980</v>
       </c>
       <c r="D34" t="s">
-        <v>67</v>
+        <v>93</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>68</v>
-      </c>
-      <c r="B35">
-        <v>2013</v>
+        <v>94</v>
+      </c>
+      <c r="B35" t="s">
+        <v>72</v>
       </c>
       <c r="C35">
         <v>161803</v>
       </c>
       <c r="D35" t="s">
-        <v>69</v>
+        <v>95</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>70</v>
-      </c>
-      <c r="B36">
-        <v>2022</v>
+        <v>96</v>
+      </c>
+      <c r="B36" t="s">
+        <v>23</v>
       </c>
       <c r="C36">
         <v>1043816</v>
       </c>
       <c r="D36" t="s">
-        <v>71</v>
+        <v>97</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>72</v>
-      </c>
-      <c r="B37">
-        <v>2005</v>
+        <v>98</v>
+      </c>
+      <c r="B37" t="s">
+        <v>62</v>
       </c>
       <c r="C37">
         <v>13015</v>
       </c>
       <c r="D37" t="s">
-        <v>73</v>
+        <v>99</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>74</v>
-      </c>
-      <c r="B38">
-        <v>1993</v>
+        <v>100</v>
+      </c>
+      <c r="B38" t="s">
+        <v>101</v>
       </c>
       <c r="C38">
         <v>25117</v>
       </c>
       <c r="D38" t="s">
-        <v>75</v>
+        <v>102</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>76</v>
-      </c>
-      <c r="B39">
-        <v>2007</v>
+        <v>103</v>
+      </c>
+      <c r="B39" t="s">
+        <v>104</v>
       </c>
       <c r="C39">
         <v>24447</v>
       </c>
       <c r="D39" t="s">
-        <v>77</v>
+        <v>105</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>78</v>
-      </c>
-      <c r="B40">
-        <v>2006</v>
+        <v>106</v>
+      </c>
+      <c r="B40" t="s">
+        <v>80</v>
       </c>
       <c r="C40">
         <v>34515</v>
       </c>
       <c r="D40" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>80</v>
-      </c>
-      <c r="B41">
-        <v>2026</v>
+        <v>108</v>
+      </c>
+      <c r="B41" t="s">
+        <v>20</v>
       </c>
       <c r="C41">
         <v>1632879</v>
       </c>
       <c r="D41" t="s">
-        <v>81</v>
+        <v>109</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>82</v>
-      </c>
-      <c r="B42">
-        <v>2011</v>
+        <v>110</v>
+      </c>
+      <c r="B42" t="s">
+        <v>51</v>
       </c>
       <c r="C42">
         <v>80379</v>
       </c>
       <c r="D42" t="s">
-        <v>83</v>
+        <v>111</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>84</v>
-      </c>
-      <c r="B43">
-        <v>2025</v>
+        <v>112</v>
+      </c>
+      <c r="B43" t="s">
+        <v>113</v>
       </c>
       <c r="C43">
         <v>1547831</v>
       </c>
       <c r="D43" t="s">
-        <v>85</v>
+        <v>114</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>86</v>
-      </c>
-      <c r="B44">
-        <v>1996</v>
+        <v>115</v>
+      </c>
+      <c r="B44" t="s">
+        <v>59</v>
       </c>
       <c r="C44">
         <v>18128</v>
       </c>
       <c r="D44" t="s">
-        <v>87</v>
+        <v>116</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>88</v>
-      </c>
-      <c r="B45">
-        <v>2023</v>
+        <v>117</v>
+      </c>
+      <c r="B45" t="s">
+        <v>54</v>
       </c>
       <c r="C45">
         <v>1121692</v>
       </c>
       <c r="D45" t="s">
-        <v>89</v>
+        <v>118</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>90</v>
-      </c>
-      <c r="B46">
-        <v>2013</v>
+        <v>119</v>
+      </c>
+      <c r="B46" t="s">
+        <v>72</v>
       </c>
       <c r="C46">
         <v>185574</v>
       </c>
       <c r="D46" t="s">
-        <v>91</v>
+        <v>120</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>92</v>
-      </c>
-      <c r="B47">
-        <v>2002</v>
+        <v>121</v>
+      </c>
+      <c r="B47" t="s">
+        <v>122</v>
       </c>
       <c r="C47">
         <v>20211</v>
       </c>
       <c r="D47" t="s">
-        <v>93</v>
+        <v>123</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>94</v>
-      </c>
-      <c r="B48">
-        <v>2001</v>
+        <v>124</v>
+      </c>
+      <c r="B48" t="s">
+        <v>125</v>
       </c>
       <c r="C48">
         <v>20679</v>
       </c>
       <c r="D48" t="s">
-        <v>95</v>
+        <v>126</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>96</v>
-      </c>
-      <c r="B49">
-        <v>2024</v>
+        <v>127</v>
+      </c>
+      <c r="B49" t="s">
+        <v>34</v>
       </c>
       <c r="C49">
         <v>1255883</v>
       </c>
       <c r="D49" t="s">
-        <v>97</v>
+        <v>128</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>98</v>
-      </c>
-      <c r="B50">
-        <v>2013</v>
+        <v>129</v>
+      </c>
+      <c r="B50" t="s">
+        <v>72</v>
       </c>
       <c r="C50">
         <v>216652</v>
       </c>
       <c r="D50" t="s">
-        <v>99</v>
+        <v>130</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>100</v>
-      </c>
-      <c r="B51">
-        <v>2024</v>
+        <v>131</v>
+      </c>
+      <c r="B51" t="s">
+        <v>34</v>
       </c>
       <c r="C51">
         <v>1245157</v>
       </c>
       <c r="D51" t="s">
-        <v>101</v>
+        <v>132</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>102</v>
-      </c>
-      <c r="B52">
-        <v>2017</v>
+        <v>133</v>
+      </c>
+      <c r="B52" t="s">
+        <v>69</v>
       </c>
       <c r="C52">
         <v>454787</v>
       </c>
       <c r="D52" t="s">
-        <v>103</v>
+        <v>134</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>104</v>
-      </c>
-      <c r="B53">
-        <v>2020</v>
+        <v>135</v>
+      </c>
+      <c r="B53" t="s">
+        <v>5</v>
       </c>
       <c r="C53">
         <v>767809</v>
       </c>
       <c r="D53" t="s">
-        <v>105</v>
+        <v>136</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>106</v>
-      </c>
-      <c r="B54">
-        <v>2008</v>
+        <v>137</v>
+      </c>
+      <c r="B54" t="s">
+        <v>17</v>
       </c>
       <c r="C54">
         <v>32836</v>
       </c>
       <c r="D54" t="s">
-        <v>107</v>
+        <v>138</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>108</v>
-      </c>
-      <c r="B55">
-        <v>2023</v>
+        <v>139</v>
+      </c>
+      <c r="B55" t="s">
+        <v>54</v>
       </c>
       <c r="C55">
         <v>1179829</v>
       </c>
       <c r="D55" t="s">
-        <v>109</v>
+        <v>140</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>110</v>
-      </c>
-      <c r="B56">
-        <v>2026</v>
+        <v>141</v>
+      </c>
+      <c r="B56" t="s">
+        <v>20</v>
       </c>
       <c r="C56">
         <v>1664894</v>
       </c>
       <c r="D56" t="s">
-        <v>111</v>
+        <v>142</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>112</v>
-      </c>
-      <c r="B57">
-        <v>2019</v>
+        <v>143</v>
+      </c>
+      <c r="B57" t="s">
+        <v>8</v>
       </c>
       <c r="C57">
         <v>627016</v>
       </c>
       <c r="D57" t="s">
-        <v>113</v>
+        <v>144</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>114</v>
-      </c>
-      <c r="B58">
-        <v>2017</v>
+        <v>145</v>
+      </c>
+      <c r="B58" t="s">
+        <v>69</v>
       </c>
       <c r="C58">
         <v>488223</v>
       </c>
       <c r="D58" t="s">
-        <v>115</v>
+        <v>146</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>116</v>
-      </c>
-      <c r="B59">
-        <v>1990</v>
+        <v>147</v>
+      </c>
+      <c r="B59" t="s">
+        <v>148</v>
       </c>
       <c r="C59">
         <v>25160</v>
       </c>
       <c r="D59" t="s">
-        <v>117</v>
+        <v>149</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>118</v>
-      </c>
-      <c r="B60">
-        <v>2019</v>
+        <v>150</v>
+      </c>
+      <c r="B60" t="s">
+        <v>8</v>
       </c>
       <c r="C60">
         <v>586247</v>
       </c>
       <c r="D60" t="s">
-        <v>119</v>
+        <v>151</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>120</v>
-      </c>
-      <c r="B61">
-        <v>2020</v>
+        <v>152</v>
+      </c>
+      <c r="B61" t="s">
+        <v>5</v>
       </c>
       <c r="C61">
         <v>638706</v>
       </c>
       <c r="D61" t="s">
-        <v>121</v>
+        <v>153</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>122</v>
-      </c>
-      <c r="B62">
-        <v>2020</v>
+        <v>154</v>
+      </c>
+      <c r="B62" t="s">
+        <v>5</v>
       </c>
       <c r="C62">
         <v>675929</v>
       </c>
       <c r="D62" t="s">
-        <v>123</v>
+        <v>155</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>124</v>
-      </c>
-      <c r="B63">
-        <v>1989</v>
+        <v>156</v>
+      </c>
+      <c r="B63" t="s">
+        <v>157</v>
       </c>
       <c r="C63">
         <v>14733</v>
       </c>
       <c r="D63" t="s">
-        <v>125</v>
+        <v>158</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>126</v>
-      </c>
-      <c r="B64">
-        <v>2020</v>
+        <v>159</v>
+      </c>
+      <c r="B64" t="s">
+        <v>5</v>
       </c>
       <c r="C64">
         <v>753702</v>
       </c>
       <c r="D64" t="s">
-        <v>127</v>
+        <v>160</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>128</v>
-      </c>
-      <c r="B65">
-        <v>1999</v>
+        <v>161</v>
+      </c>
+      <c r="B65" t="s">
+        <v>48</v>
       </c>
       <c r="C65">
         <v>17870</v>
       </c>
       <c r="D65" t="s">
-        <v>129</v>
+        <v>162</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>130</v>
-      </c>
-      <c r="B66">
-        <v>2010</v>
+        <v>163</v>
+      </c>
+      <c r="B66" t="s">
+        <v>90</v>
       </c>
       <c r="C66">
         <v>46967</v>
       </c>
       <c r="D66" t="s">
-        <v>131</v>
+        <v>164</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>132</v>
-      </c>
-      <c r="B67">
-        <v>1983</v>
+        <v>165</v>
+      </c>
+      <c r="B67" t="s">
+        <v>166</v>
       </c>
       <c r="C67">
         <v>21585</v>
       </c>
       <c r="D67" t="s">
-        <v>133</v>
+        <v>167</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>134</v>
-      </c>
-      <c r="B68">
-        <v>2023</v>
+        <v>168</v>
+      </c>
+      <c r="B68" t="s">
+        <v>54</v>
       </c>
       <c r="C68">
         <v>1199400</v>
       </c>
       <c r="D68" t="s">
-        <v>135</v>
+        <v>169</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>136</v>
-      </c>
-      <c r="B69">
-        <v>1983</v>
+        <v>170</v>
+      </c>
+      <c r="B69" t="s">
+        <v>166</v>
       </c>
       <c r="C69">
         <v>15251</v>
       </c>
       <c r="D69" t="s">
-        <v>137</v>
+        <v>171</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>138</v>
-      </c>
-      <c r="B70">
-        <v>2022</v>
+        <v>172</v>
+      </c>
+      <c r="B70" t="s">
+        <v>23</v>
       </c>
       <c r="C70">
         <v>975088</v>
       </c>
       <c r="D70" t="s">
-        <v>139</v>
+        <v>173</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>140</v>
-      </c>
-      <c r="B71">
-        <v>1982</v>
+        <v>174</v>
+      </c>
+      <c r="B71" t="s">
+        <v>175</v>
       </c>
       <c r="C71">
         <v>21923</v>
       </c>
       <c r="D71" t="s">
-        <v>141</v>
+        <v>176</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>142</v>
-      </c>
-      <c r="B72">
-        <v>2025</v>
+        <v>177</v>
+      </c>
+      <c r="B72" t="s">
+        <v>113</v>
       </c>
       <c r="C72">
         <v>1564460</v>
       </c>
       <c r="D72" t="s">
-        <v>143</v>
+        <v>178</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
+        <v>179</v>
+      </c>
+      <c r="B73" t="s">
+        <v>90</v>
+      </c>
+      <c r="C73">
+        <v>49505</v>
+      </c>
+      <c r="D73" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
+        <v>181</v>
+      </c>
+      <c r="B74" t="s">
+        <v>54</v>
+      </c>
+      <c r="C74">
+        <v>1169007</v>
+      </c>
+      <c r="D74" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
+        <v>183</v>
+      </c>
+      <c r="B75" t="s">
+        <v>23</v>
+      </c>
+      <c r="C75">
+        <v>1024961</v>
+      </c>
+      <c r="D75" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
+        <v>185</v>
+      </c>
+      <c r="B76" t="s">
+        <v>8</v>
+      </c>
+      <c r="C76">
+        <v>642739</v>
+      </c>
+      <c r="D76" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
+        <v>187</v>
+      </c>
+      <c r="B77" t="s">
+        <v>188</v>
+      </c>
+      <c r="C77">
+        <v>308571</v>
+      </c>
+      <c r="D77" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
+        <v>190</v>
+      </c>
+      <c r="B78" t="s">
+        <v>5</v>
+      </c>
+      <c r="C78">
+        <v>701687</v>
+      </c>
+      <c r="D78" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
+        <v>192</v>
+      </c>
+      <c r="B79" t="s">
+        <v>193</v>
+      </c>
+      <c r="C79">
+        <v>13590</v>
+      </c>
+      <c r="D79" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
+        <v>195</v>
+      </c>
+      <c r="B80" t="s">
+        <v>14</v>
+      </c>
+      <c r="C80">
+        <v>191489</v>
+      </c>
+      <c r="D80" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
+        <v>197</v>
+      </c>
+      <c r="B81" t="s">
+        <v>198</v>
+      </c>
+      <c r="C81">
+        <v>21586</v>
+      </c>
+      <c r="D81" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
+        <v>200</v>
+      </c>
+      <c r="B82" t="s">
+        <v>80</v>
+      </c>
+      <c r="C82">
+        <v>47658</v>
+      </c>
+      <c r="D82" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
+        <v>202</v>
+      </c>
+      <c r="B83" t="s">
+        <v>23</v>
+      </c>
+      <c r="C83">
+        <v>1023901</v>
+      </c>
+      <c r="D83" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A84" t="s">
+        <v>204</v>
+      </c>
+      <c r="B84" t="s">
+        <v>69</v>
+      </c>
+      <c r="C84">
+        <v>494368</v>
+      </c>
+      <c r="D84" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
+        <v>206</v>
+      </c>
+      <c r="B85" t="s">
+        <v>54</v>
+      </c>
+      <c r="C85">
+        <v>1093247</v>
+      </c>
+      <c r="D85" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A86" t="s">
+        <v>208</v>
+      </c>
+      <c r="B86" t="s">
+        <v>54</v>
+      </c>
+      <c r="C86">
+        <v>1111585</v>
+      </c>
+      <c r="D86" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A87" t="s">
+        <v>210</v>
+      </c>
+      <c r="B87" t="s">
+        <v>5</v>
+      </c>
+      <c r="C87">
+        <v>689643</v>
+      </c>
+      <c r="D87" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
+        <v>212</v>
+      </c>
+      <c r="B88" t="s">
+        <v>45</v>
+      </c>
+      <c r="C88">
+        <v>17871</v>
+      </c>
+      <c r="D88" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A89" t="s">
+        <v>214</v>
+      </c>
+      <c r="B89" t="s">
+        <v>62</v>
+      </c>
+      <c r="C89">
+        <v>261581</v>
+      </c>
+      <c r="D89" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A90" t="s">
+        <v>216</v>
+      </c>
+      <c r="B90" t="s">
+        <v>69</v>
+      </c>
+      <c r="C90">
+        <v>444705</v>
+      </c>
+      <c r="D90" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A91" t="s">
+        <v>218</v>
+      </c>
+      <c r="B91" t="s">
+        <v>23</v>
+      </c>
+      <c r="C91">
+        <v>1054569</v>
+      </c>
+      <c r="D91" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A92" t="s">
+        <v>220</v>
+      </c>
+      <c r="B92" t="s">
+        <v>69</v>
+      </c>
+      <c r="C92">
+        <v>435351</v>
+      </c>
+      <c r="D92" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A93" t="s">
+        <v>222</v>
+      </c>
+      <c r="B93" t="s">
+        <v>54</v>
+      </c>
+      <c r="C93">
+        <v>1107516</v>
+      </c>
+      <c r="D93" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
+        <v>224</v>
+      </c>
+      <c r="B94" t="s">
+        <v>8</v>
+      </c>
+      <c r="C94">
+        <v>612392</v>
+      </c>
+      <c r="D94" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A95" t="s">
+        <v>226</v>
+      </c>
+      <c r="B95" t="s">
+        <v>5</v>
+      </c>
+      <c r="C95">
+        <v>672992</v>
+      </c>
+      <c r="D95" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A96" t="s">
+        <v>228</v>
+      </c>
+      <c r="B96" t="s">
+        <v>113</v>
+      </c>
+      <c r="C96">
+        <v>1541013</v>
+      </c>
+      <c r="D96" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A97" t="s">
+        <v>230</v>
+      </c>
+      <c r="B97" t="s">
+        <v>231</v>
+      </c>
+      <c r="C97">
+        <v>34512</v>
+      </c>
+      <c r="D97" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A98" t="s">
+        <v>233</v>
+      </c>
+      <c r="B98" t="s">
+        <v>23</v>
+      </c>
+      <c r="C98">
+        <v>1015999</v>
+      </c>
+      <c r="D98" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A99" t="s">
+        <v>235</v>
+      </c>
+      <c r="B99" t="s">
+        <v>54</v>
+      </c>
+      <c r="C99">
+        <v>1111957</v>
+      </c>
+      <c r="D99" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A100" t="s">
+        <v>237</v>
+      </c>
+      <c r="B100" t="s">
+        <v>238</v>
+      </c>
+      <c r="C100">
+        <v>24665</v>
+      </c>
+      <c r="D100" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A101" t="s">
+        <v>240</v>
+      </c>
+      <c r="B101">
+        <v>2023</v>
+      </c>
+      <c r="C101">
+        <v>1212312</v>
+      </c>
+      <c r="D101" s="2" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A102" t="s">
+        <v>242</v>
+      </c>
+      <c r="B102">
+        <v>2022</v>
+      </c>
+      <c r="C102">
+        <v>1020051</v>
+      </c>
+      <c r="D102" s="2" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A103" t="s">
+        <v>244</v>
+      </c>
+      <c r="B103">
+        <v>2024</v>
+      </c>
+      <c r="C103">
+        <v>1287248</v>
+      </c>
+      <c r="D103" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A104" t="s">
+        <v>246</v>
+      </c>
+      <c r="B104">
+        <v>2010</v>
+      </c>
+      <c r="C104">
+        <v>52252</v>
+      </c>
+      <c r="D104" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A105" t="s">
+        <v>248</v>
+      </c>
+      <c r="B105">
+        <v>2010</v>
+      </c>
+      <c r="C105">
+        <v>47911</v>
+      </c>
+      <c r="D105" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A106" t="s">
+        <v>250</v>
+      </c>
+      <c r="B106">
+        <v>2009</v>
+      </c>
+      <c r="C106">
+        <v>26621</v>
+      </c>
+      <c r="D106" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A107" t="s">
+        <v>252</v>
+      </c>
+      <c r="B107">
+        <v>2012</v>
+      </c>
+      <c r="C107">
+        <v>110549</v>
+      </c>
+      <c r="D107" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A108" t="s">
+        <v>254</v>
+      </c>
+      <c r="B108">
+        <v>2017</v>
+      </c>
+      <c r="C108">
+        <v>456193</v>
+      </c>
+      <c r="D108" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A109" t="s">
+        <v>256</v>
+      </c>
+      <c r="B109">
+        <v>2022</v>
+      </c>
+      <c r="C109">
+        <v>937348</v>
+      </c>
+      <c r="D109" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A110" t="s">
+        <v>258</v>
+      </c>
+      <c r="B110">
+        <v>2017</v>
+      </c>
+      <c r="C110">
+        <v>484413</v>
+      </c>
+      <c r="D110" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A111" t="s">
+        <v>260</v>
+      </c>
+      <c r="B111">
+        <v>2003</v>
+      </c>
+      <c r="C111">
+        <v>198306</v>
+      </c>
+      <c r="D111" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A112" t="s">
+        <v>262</v>
+      </c>
+      <c r="B112">
+        <v>2017</v>
+      </c>
+      <c r="C112">
+        <v>442087</v>
+      </c>
+      <c r="D112" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A113" t="s">
+        <v>264</v>
+      </c>
+      <c r="B113">
+        <v>2012</v>
+      </c>
+      <c r="C113">
+        <v>84154</v>
+      </c>
+      <c r="D113" t="s">
+        <v>265</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D101" r:id="rId1" xr:uid="{419420B0-79EB-44E4-B02A-6B12850B061F}"/>
+    <hyperlink ref="D102" r:id="rId2" xr:uid="{7B2A5A40-BC38-4883-8EB3-BC0C9A5C6138}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updating to use the new billion dollar list
</commit_message>
<xml_diff>
--- a/Comedy_Whitelist.xlsx
+++ b/Comedy_Whitelist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bigba\aa Personal Projects\Letterboxd-List-Scraping\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6FA3610-C400-42EF-B278-8D88400C211F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B42148C-FAA6-4007-93DA-CBC3DD5FE732}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="278">
   <si>
     <t>Title</t>
   </si>
@@ -130,12 +130,6 @@
     <t>https://letterboxd.com/film/stand-up-solutions/</t>
   </si>
   <si>
-    <t>08:46:00</t>
-  </si>
-  <si>
-    <t>https://letterboxd.com/film/8-46-2020/</t>
-  </si>
-  <si>
     <t>John Mulaney: The Comeback Kid</t>
   </si>
   <si>
@@ -205,120 +199,114 @@
     <t>https://letterboxd.com/film/george-carlin-back-in-town/</t>
   </si>
   <si>
-    <t>One Night Stand: Flight of the Conchords</t>
+    <t>Rowan Atkinson Live</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/rowan-atkinson-live/</t>
+  </si>
+  <si>
+    <t>Flight of the Conchords: Live in London</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/flight-of-the-conchords-live-in-london/</t>
+  </si>
+  <si>
+    <t>Hasan Minhaj: Homecoming King</t>
+  </si>
+  <si>
+    <t>2017</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/hasan-minhaj-homecoming-king/</t>
+  </si>
+  <si>
+    <t>Bo Burnham: What.</t>
+  </si>
+  <si>
+    <t>2013</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/bo-burnham-what/</t>
+  </si>
+  <si>
+    <t>Richard Pryor: Live in Concert</t>
+  </si>
+  <si>
+    <t>1979</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/richard-pryor-live-in-concert/</t>
+  </si>
+  <si>
+    <t>George Carlin: You Are All Diseased</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/george-carlin-you-are-all-diseased/</t>
+  </si>
+  <si>
+    <t>Bill Hicks: Relentless</t>
+  </si>
+  <si>
+    <t>2006</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/bill-hicks-relentless/</t>
+  </si>
+  <si>
+    <t>Louis C.K.: Chewed Up</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/louis-ck-chewed-up/</t>
+  </si>
+  <si>
+    <t>Shane Gillis: Live in Austin</t>
+  </si>
+  <si>
+    <t>2021</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/shane-gillis-live-in-austin/</t>
+  </si>
+  <si>
+    <t>George Carlin: Itâ€TMs Bad for Ya!</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/george-carlin-its-bad-for-ya/</t>
+  </si>
+  <si>
+    <t>Louis C.K.: Hilarious</t>
+  </si>
+  <si>
+    <t>2010</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/louis-ck-hilarious/</t>
+  </si>
+  <si>
+    <t>Jacqueline Novak: Get on Your Knees</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/jacqueline-novak-get-on-your-knees/</t>
+  </si>
+  <si>
+    <t>CM101MMXI Fundamentals</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/cm101mmxi-fundamentals/</t>
+  </si>
+  <si>
+    <t>Panayotis Pascot: Almost</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/panayotis-pascot-almost/</t>
+  </si>
+  <si>
+    <t>George Carlin: Life Is Worth Losing</t>
   </si>
   <si>
     <t>2005</t>
   </si>
   <si>
-    <t>https://letterboxd.com/film/one-night-stand-flight-of-the-conchords/</t>
-  </si>
-  <si>
-    <t>Rowan Atkinson Live</t>
-  </si>
-  <si>
-    <t>https://letterboxd.com/film/rowan-atkinson-live/</t>
-  </si>
-  <si>
-    <t>Flight of the Conchords: Live in London</t>
-  </si>
-  <si>
-    <t>https://letterboxd.com/film/flight-of-the-conchords-live-in-london/</t>
-  </si>
-  <si>
-    <t>Hasan Minhaj: Homecoming King</t>
-  </si>
-  <si>
-    <t>2017</t>
-  </si>
-  <si>
-    <t>https://letterboxd.com/film/hasan-minhaj-homecoming-king/</t>
-  </si>
-  <si>
-    <t>Bo Burnham: What.</t>
-  </si>
-  <si>
-    <t>2013</t>
-  </si>
-  <si>
-    <t>https://letterboxd.com/film/bo-burnham-what/</t>
-  </si>
-  <si>
-    <t>Richard Pryor: Live in Concert</t>
-  </si>
-  <si>
-    <t>1979</t>
-  </si>
-  <si>
-    <t>https://letterboxd.com/film/richard-pryor-live-in-concert/</t>
-  </si>
-  <si>
-    <t>George Carlin: You Are All Diseased</t>
-  </si>
-  <si>
-    <t>https://letterboxd.com/film/george-carlin-you-are-all-diseased/</t>
-  </si>
-  <si>
-    <t>Bill Hicks: Relentless</t>
-  </si>
-  <si>
-    <t>2006</t>
-  </si>
-  <si>
-    <t>https://letterboxd.com/film/bill-hicks-relentless/</t>
-  </si>
-  <si>
-    <t>Louis C.K.: Chewed Up</t>
-  </si>
-  <si>
-    <t>https://letterboxd.com/film/louis-ck-chewed-up/</t>
-  </si>
-  <si>
-    <t>Shane Gillis: Live in Austin</t>
-  </si>
-  <si>
-    <t>2021</t>
-  </si>
-  <si>
-    <t>https://letterboxd.com/film/shane-gillis-live-in-austin/</t>
-  </si>
-  <si>
-    <t>George Carlin: Itâ€TMs Bad for Ya!</t>
-  </si>
-  <si>
-    <t>https://letterboxd.com/film/george-carlin-its-bad-for-ya/</t>
-  </si>
-  <si>
-    <t>Louis C.K.: Hilarious</t>
-  </si>
-  <si>
-    <t>2010</t>
-  </si>
-  <si>
-    <t>https://letterboxd.com/film/louis-ck-hilarious/</t>
-  </si>
-  <si>
-    <t>Jacqueline Novak: Get on Your Knees</t>
-  </si>
-  <si>
-    <t>https://letterboxd.com/film/jacqueline-novak-get-on-your-knees/</t>
-  </si>
-  <si>
-    <t>CM101MMXI Fundamentals</t>
-  </si>
-  <si>
-    <t>https://letterboxd.com/film/cm101mmxi-fundamentals/</t>
-  </si>
-  <si>
-    <t>Panayotis Pascot: Almost</t>
-  </si>
-  <si>
-    <t>https://letterboxd.com/film/panayotis-pascot-almost/</t>
-  </si>
-  <si>
-    <t>George Carlin: Life Is Worth Losing</t>
-  </si>
-  <si>
     <t>https://letterboxd.com/film/george-carlin-life-is-worth-losing/</t>
   </si>
   <si>
@@ -664,12 +652,6 @@
     <t>https://letterboxd.com/film/chris-rock-never-scared/</t>
   </si>
   <si>
-    <t>Louis C.K.: One Night Stand</t>
-  </si>
-  <si>
-    <t>https://letterboxd.com/film/louis-ck-one-night-stand/</t>
-  </si>
-  <si>
     <t>Dave Chappelle: The Age of Spin</t>
   </si>
   <si>
@@ -775,6 +757,9 @@
     <t>Robin Williams: Weapons of Self Destruction</t>
   </si>
   <si>
+    <t>2009</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/robin-williams-weapons-of-self-destruction/</t>
   </si>
   <si>
@@ -784,7 +769,7 @@
     <t>https://letterboxd.com/film/hannibal-buress-animal-furnace/</t>
   </si>
   <si>
-    <t>Norm Macdonald: Hitlerâ€™s Dog, Gossip &amp; Trickery</t>
+    <t>Norm Macdonald: Hitlerâ€TMs Dog, Gossip &amp; Trickery</t>
   </si>
   <si>
     <t>https://letterboxd.com/film/norm-macdonald-hitlers-dog-gossip-trickery/</t>
@@ -805,6 +790,9 @@
     <t>Ricky Gervais Live: Animals</t>
   </si>
   <si>
+    <t>2003</t>
+  </si>
+  <si>
     <t>https://letterboxd.com/film/ricky-gervais-live-animals/</t>
   </si>
   <si>
@@ -818,6 +806,54 @@
   </si>
   <si>
     <t>https://letterboxd.com/film/donald-glover-weirdo/</t>
+  </si>
+  <si>
+    <t>Dan and Phil: Terrible Influence</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/dan-and-phil-terrible-influence/</t>
+  </si>
+  <si>
+    <t>Ricky Jay and His 52 Assistants</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/ricky-jay-and-his-52-assistants/</t>
+  </si>
+  <si>
+    <t>Dan and Philâ€TMs The Amazing Tour is Not on Fire</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-amazing-tour-is-not-on-fire/</t>
+  </si>
+  <si>
+    <t>Interactive Introverts</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/interactive-introverts/</t>
+  </si>
+  <si>
+    <t>The Mighty Boosh Live</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-mighty-boosh-live/</t>
+  </si>
+  <si>
+    <t>Bigger! With Brennan and Izzy</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/bigger-with-brennan-and-izzy/</t>
+  </si>
+  <si>
+    <t>Eddie Murphy Raw</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/eddie-murphy-raw/</t>
+  </si>
+  <si>
+    <t>Bo Burnham: Inside</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/bo-burnham-inside/</t>
   </si>
 </sst>
 </file>
@@ -1191,7 +1227,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D113"/>
+  <dimension ref="A1:D118"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
@@ -1367,94 +1403,94 @@
         <v>36</v>
       </c>
       <c r="B13" t="s">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="C13">
-        <v>714842</v>
+        <v>367735</v>
       </c>
       <c r="D13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B14" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C14">
-        <v>367735</v>
+        <v>25161</v>
       </c>
       <c r="D14" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B15" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C15">
-        <v>25161</v>
+        <v>20147</v>
       </c>
       <c r="D15" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C16">
-        <v>20147</v>
+        <v>13589</v>
       </c>
       <c r="D16" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B17" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C17">
-        <v>13589</v>
+        <v>60233</v>
       </c>
       <c r="D17" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B18" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C18">
-        <v>60233</v>
+        <v>1179932</v>
       </c>
       <c r="D18" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B19" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="C19">
-        <v>1179932</v>
+        <v>57469</v>
       </c>
       <c r="D19" t="s">
         <v>55</v>
@@ -1465,24 +1501,24 @@
         <v>56</v>
       </c>
       <c r="B20" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="C20">
-        <v>57469</v>
+        <v>34509</v>
       </c>
       <c r="D20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B21" t="s">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="C21">
-        <v>34509</v>
+        <v>18458</v>
       </c>
       <c r="D21" t="s">
         <v>60</v>
@@ -1493,24 +1529,24 @@
         <v>61</v>
       </c>
       <c r="B22" t="s">
+        <v>29</v>
+      </c>
+      <c r="C22">
+        <v>550416</v>
+      </c>
+      <c r="D22" t="s">
         <v>62</v>
-      </c>
-      <c r="C22">
-        <v>147502</v>
-      </c>
-      <c r="D22" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
+        <v>63</v>
+      </c>
+      <c r="B23" t="s">
         <v>64</v>
       </c>
-      <c r="B23" t="s">
-        <v>42</v>
-      </c>
       <c r="C23">
-        <v>18458</v>
+        <v>458310</v>
       </c>
       <c r="D23" t="s">
         <v>65</v>
@@ -1521,38 +1557,38 @@
         <v>66</v>
       </c>
       <c r="B24" t="s">
-        <v>29</v>
+        <v>67</v>
       </c>
       <c r="C24">
-        <v>550416</v>
+        <v>244001</v>
       </c>
       <c r="D24" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B25" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C25">
-        <v>458310</v>
+        <v>22975</v>
       </c>
       <c r="D25" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B26" t="s">
-        <v>72</v>
+        <v>46</v>
       </c>
       <c r="C26">
-        <v>244001</v>
+        <v>34513</v>
       </c>
       <c r="D26" t="s">
         <v>73</v>
@@ -1566,7 +1602,7 @@
         <v>75</v>
       </c>
       <c r="C27">
-        <v>22975</v>
+        <v>34505</v>
       </c>
       <c r="D27" t="s">
         <v>76</v>
@@ -1577,10 +1613,10 @@
         <v>77</v>
       </c>
       <c r="B28" t="s">
-        <v>48</v>
+        <v>17</v>
       </c>
       <c r="C28">
-        <v>34513</v>
+        <v>30969</v>
       </c>
       <c r="D28" t="s">
         <v>78</v>
@@ -1594,7 +1630,7 @@
         <v>80</v>
       </c>
       <c r="C29">
-        <v>34505</v>
+        <v>872209</v>
       </c>
       <c r="D29" t="s">
         <v>81</v>
@@ -1608,7 +1644,7 @@
         <v>17</v>
       </c>
       <c r="C30">
-        <v>30969</v>
+        <v>13643</v>
       </c>
       <c r="D30" t="s">
         <v>83</v>
@@ -1622,7 +1658,7 @@
         <v>85</v>
       </c>
       <c r="C31">
-        <v>872209</v>
+        <v>45523</v>
       </c>
       <c r="D31" t="s">
         <v>86</v>
@@ -1633,10 +1669,10 @@
         <v>87</v>
       </c>
       <c r="B32" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="C32">
-        <v>13643</v>
+        <v>1214980</v>
       </c>
       <c r="D32" t="s">
         <v>88</v>
@@ -1647,38 +1683,38 @@
         <v>89</v>
       </c>
       <c r="B33" t="s">
+        <v>67</v>
+      </c>
+      <c r="C33">
+        <v>161803</v>
+      </c>
+      <c r="D33" t="s">
         <v>90</v>
-      </c>
-      <c r="C33">
-        <v>45523</v>
-      </c>
-      <c r="D33" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
+        <v>91</v>
+      </c>
+      <c r="B34" t="s">
+        <v>23</v>
+      </c>
+      <c r="C34">
+        <v>1043816</v>
+      </c>
+      <c r="D34" t="s">
         <v>92</v>
-      </c>
-      <c r="B34" t="s">
-        <v>34</v>
-      </c>
-      <c r="C34">
-        <v>1214980</v>
-      </c>
-      <c r="D34" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
+        <v>93</v>
+      </c>
+      <c r="B35" t="s">
         <v>94</v>
       </c>
-      <c r="B35" t="s">
-        <v>72</v>
-      </c>
       <c r="C35">
-        <v>161803</v>
+        <v>13015</v>
       </c>
       <c r="D35" t="s">
         <v>95</v>
@@ -1689,52 +1725,52 @@
         <v>96</v>
       </c>
       <c r="B36" t="s">
-        <v>23</v>
+        <v>97</v>
       </c>
       <c r="C36">
-        <v>1043816</v>
+        <v>25117</v>
       </c>
       <c r="D36" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B37" t="s">
-        <v>62</v>
+        <v>100</v>
       </c>
       <c r="C37">
-        <v>13015</v>
+        <v>24447</v>
       </c>
       <c r="D37" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B38" t="s">
-        <v>101</v>
+        <v>75</v>
       </c>
       <c r="C38">
-        <v>25117</v>
+        <v>34515</v>
       </c>
       <c r="D38" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B39" t="s">
-        <v>104</v>
+        <v>20</v>
       </c>
       <c r="C39">
-        <v>24447</v>
+        <v>1632879</v>
       </c>
       <c r="D39" t="s">
         <v>105</v>
@@ -1745,10 +1781,10 @@
         <v>106</v>
       </c>
       <c r="B40" t="s">
-        <v>80</v>
+        <v>49</v>
       </c>
       <c r="C40">
-        <v>34515</v>
+        <v>80379</v>
       </c>
       <c r="D40" t="s">
         <v>107</v>
@@ -1759,38 +1795,38 @@
         <v>108</v>
       </c>
       <c r="B41" t="s">
-        <v>20</v>
+        <v>109</v>
       </c>
       <c r="C41">
-        <v>1632879</v>
+        <v>1547831</v>
       </c>
       <c r="D41" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B42" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="C42">
-        <v>80379</v>
+        <v>18128</v>
       </c>
       <c r="D42" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B43" t="s">
-        <v>113</v>
+        <v>52</v>
       </c>
       <c r="C43">
-        <v>1547831</v>
+        <v>1121692</v>
       </c>
       <c r="D43" t="s">
         <v>114</v>
@@ -1801,10 +1837,10 @@
         <v>115</v>
       </c>
       <c r="B44" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="C44">
-        <v>18128</v>
+        <v>185574</v>
       </c>
       <c r="D44" t="s">
         <v>116</v>
@@ -1815,52 +1851,52 @@
         <v>117</v>
       </c>
       <c r="B45" t="s">
-        <v>54</v>
+        <v>118</v>
       </c>
       <c r="C45">
-        <v>1121692</v>
+        <v>20211</v>
       </c>
       <c r="D45" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B46" t="s">
-        <v>72</v>
+        <v>121</v>
       </c>
       <c r="C46">
-        <v>185574</v>
+        <v>20679</v>
       </c>
       <c r="D46" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B47" t="s">
-        <v>122</v>
+        <v>34</v>
       </c>
       <c r="C47">
-        <v>20211</v>
+        <v>1255883</v>
       </c>
       <c r="D47" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B48" t="s">
-        <v>125</v>
+        <v>67</v>
       </c>
       <c r="C48">
-        <v>20679</v>
+        <v>216652</v>
       </c>
       <c r="D48" t="s">
         <v>126</v>
@@ -1874,7 +1910,7 @@
         <v>34</v>
       </c>
       <c r="C49">
-        <v>1255883</v>
+        <v>1245157</v>
       </c>
       <c r="D49" t="s">
         <v>128</v>
@@ -1885,10 +1921,10 @@
         <v>129</v>
       </c>
       <c r="B50" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="C50">
-        <v>216652</v>
+        <v>454787</v>
       </c>
       <c r="D50" t="s">
         <v>130</v>
@@ -1899,10 +1935,10 @@
         <v>131</v>
       </c>
       <c r="B51" t="s">
-        <v>34</v>
+        <v>5</v>
       </c>
       <c r="C51">
-        <v>1245157</v>
+        <v>767809</v>
       </c>
       <c r="D51" t="s">
         <v>132</v>
@@ -1913,10 +1949,10 @@
         <v>133</v>
       </c>
       <c r="B52" t="s">
-        <v>69</v>
+        <v>17</v>
       </c>
       <c r="C52">
-        <v>454787</v>
+        <v>32836</v>
       </c>
       <c r="D52" t="s">
         <v>134</v>
@@ -1927,10 +1963,10 @@
         <v>135</v>
       </c>
       <c r="B53" t="s">
-        <v>5</v>
+        <v>52</v>
       </c>
       <c r="C53">
-        <v>767809</v>
+        <v>1179829</v>
       </c>
       <c r="D53" t="s">
         <v>136</v>
@@ -1941,10 +1977,10 @@
         <v>137</v>
       </c>
       <c r="B54" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C54">
-        <v>32836</v>
+        <v>1664894</v>
       </c>
       <c r="D54" t="s">
         <v>138</v>
@@ -1955,10 +1991,10 @@
         <v>139</v>
       </c>
       <c r="B55" t="s">
-        <v>54</v>
+        <v>8</v>
       </c>
       <c r="C55">
-        <v>1179829</v>
+        <v>627016</v>
       </c>
       <c r="D55" t="s">
         <v>140</v>
@@ -1969,10 +2005,10 @@
         <v>141</v>
       </c>
       <c r="B56" t="s">
-        <v>20</v>
+        <v>64</v>
       </c>
       <c r="C56">
-        <v>1664894</v>
+        <v>488223</v>
       </c>
       <c r="D56" t="s">
         <v>142</v>
@@ -1983,38 +2019,38 @@
         <v>143</v>
       </c>
       <c r="B57" t="s">
-        <v>8</v>
+        <v>144</v>
       </c>
       <c r="C57">
-        <v>627016</v>
+        <v>25160</v>
       </c>
       <c r="D57" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B58" t="s">
-        <v>69</v>
+        <v>8</v>
       </c>
       <c r="C58">
-        <v>488223</v>
+        <v>586247</v>
       </c>
       <c r="D58" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B59" t="s">
-        <v>148</v>
+        <v>5</v>
       </c>
       <c r="C59">
-        <v>25160</v>
+        <v>638706</v>
       </c>
       <c r="D59" t="s">
         <v>149</v>
@@ -2025,10 +2061,10 @@
         <v>150</v>
       </c>
       <c r="B60" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C60">
-        <v>586247</v>
+        <v>675929</v>
       </c>
       <c r="D60" t="s">
         <v>151</v>
@@ -2039,38 +2075,38 @@
         <v>152</v>
       </c>
       <c r="B61" t="s">
-        <v>5</v>
+        <v>153</v>
       </c>
       <c r="C61">
-        <v>638706</v>
+        <v>14733</v>
       </c>
       <c r="D61" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B62" t="s">
         <v>5</v>
       </c>
       <c r="C62">
-        <v>675929</v>
+        <v>753702</v>
       </c>
       <c r="D62" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B63" t="s">
-        <v>157</v>
+        <v>46</v>
       </c>
       <c r="C63">
-        <v>14733</v>
+        <v>17870</v>
       </c>
       <c r="D63" t="s">
         <v>158</v>
@@ -2081,10 +2117,10 @@
         <v>159</v>
       </c>
       <c r="B64" t="s">
-        <v>5</v>
+        <v>85</v>
       </c>
       <c r="C64">
-        <v>753702</v>
+        <v>46967</v>
       </c>
       <c r="D64" t="s">
         <v>160</v>
@@ -2095,38 +2131,38 @@
         <v>161</v>
       </c>
       <c r="B65" t="s">
-        <v>48</v>
+        <v>162</v>
       </c>
       <c r="C65">
-        <v>17870</v>
+        <v>21585</v>
       </c>
       <c r="D65" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B66" t="s">
-        <v>90</v>
+        <v>52</v>
       </c>
       <c r="C66">
-        <v>46967</v>
+        <v>1199400</v>
       </c>
       <c r="D66" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B67" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="C67">
-        <v>21585</v>
+        <v>15251</v>
       </c>
       <c r="D67" t="s">
         <v>167</v>
@@ -2137,10 +2173,10 @@
         <v>168</v>
       </c>
       <c r="B68" t="s">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="C68">
-        <v>1199400</v>
+        <v>975088</v>
       </c>
       <c r="D68" t="s">
         <v>169</v>
@@ -2151,38 +2187,38 @@
         <v>170</v>
       </c>
       <c r="B69" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="C69">
-        <v>15251</v>
+        <v>21923</v>
       </c>
       <c r="D69" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B70" t="s">
-        <v>23</v>
+        <v>109</v>
       </c>
       <c r="C70">
-        <v>975088</v>
+        <v>1564460</v>
       </c>
       <c r="D70" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B71" t="s">
-        <v>175</v>
+        <v>85</v>
       </c>
       <c r="C71">
-        <v>21923</v>
+        <v>49505</v>
       </c>
       <c r="D71" t="s">
         <v>176</v>
@@ -2193,10 +2229,10 @@
         <v>177</v>
       </c>
       <c r="B72" t="s">
-        <v>113</v>
+        <v>52</v>
       </c>
       <c r="C72">
-        <v>1564460</v>
+        <v>1169007</v>
       </c>
       <c r="D72" t="s">
         <v>178</v>
@@ -2207,10 +2243,10 @@
         <v>179</v>
       </c>
       <c r="B73" t="s">
-        <v>90</v>
+        <v>23</v>
       </c>
       <c r="C73">
-        <v>49505</v>
+        <v>1024961</v>
       </c>
       <c r="D73" t="s">
         <v>180</v>
@@ -2221,10 +2257,10 @@
         <v>181</v>
       </c>
       <c r="B74" t="s">
-        <v>54</v>
+        <v>8</v>
       </c>
       <c r="C74">
-        <v>1169007</v>
+        <v>642739</v>
       </c>
       <c r="D74" t="s">
         <v>182</v>
@@ -2235,94 +2271,94 @@
         <v>183</v>
       </c>
       <c r="B75" t="s">
-        <v>23</v>
+        <v>184</v>
       </c>
       <c r="C75">
-        <v>1024961</v>
+        <v>308571</v>
       </c>
       <c r="D75" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B76" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C76">
-        <v>642739</v>
+        <v>701687</v>
       </c>
       <c r="D76" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B77" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C77">
-        <v>308571</v>
+        <v>13590</v>
       </c>
       <c r="D77" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B78" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="C78">
-        <v>701687</v>
+        <v>191489</v>
       </c>
       <c r="D78" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B79" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C79">
-        <v>13590</v>
+        <v>21586</v>
       </c>
       <c r="D79" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B80" t="s">
-        <v>14</v>
+        <v>75</v>
       </c>
       <c r="C80">
-        <v>191489</v>
+        <v>47658</v>
       </c>
       <c r="D80" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B81" t="s">
-        <v>198</v>
+        <v>23</v>
       </c>
       <c r="C81">
-        <v>21586</v>
+        <v>1023901</v>
       </c>
       <c r="D81" t="s">
         <v>199</v>
@@ -2333,10 +2369,10 @@
         <v>200</v>
       </c>
       <c r="B82" t="s">
-        <v>80</v>
+        <v>64</v>
       </c>
       <c r="C82">
-        <v>47658</v>
+        <v>494368</v>
       </c>
       <c r="D82" t="s">
         <v>201</v>
@@ -2347,10 +2383,10 @@
         <v>202</v>
       </c>
       <c r="B83" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C83">
-        <v>1023901</v>
+        <v>1093247</v>
       </c>
       <c r="D83" t="s">
         <v>203</v>
@@ -2361,10 +2397,10 @@
         <v>204</v>
       </c>
       <c r="B84" t="s">
-        <v>69</v>
+        <v>52</v>
       </c>
       <c r="C84">
-        <v>494368</v>
+        <v>1111585</v>
       </c>
       <c r="D84" t="s">
         <v>205</v>
@@ -2375,10 +2411,10 @@
         <v>206</v>
       </c>
       <c r="B85" t="s">
-        <v>54</v>
+        <v>5</v>
       </c>
       <c r="C85">
-        <v>1093247</v>
+        <v>689643</v>
       </c>
       <c r="D85" t="s">
         <v>207</v>
@@ -2389,10 +2425,10 @@
         <v>208</v>
       </c>
       <c r="B86" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="C86">
-        <v>1111585</v>
+        <v>17871</v>
       </c>
       <c r="D86" t="s">
         <v>209</v>
@@ -2403,10 +2439,10 @@
         <v>210</v>
       </c>
       <c r="B87" t="s">
-        <v>5</v>
+        <v>64</v>
       </c>
       <c r="C87">
-        <v>689643</v>
+        <v>444705</v>
       </c>
       <c r="D87" t="s">
         <v>211</v>
@@ -2417,10 +2453,10 @@
         <v>212</v>
       </c>
       <c r="B88" t="s">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="C88">
-        <v>17871</v>
+        <v>1054569</v>
       </c>
       <c r="D88" t="s">
         <v>213</v>
@@ -2431,10 +2467,10 @@
         <v>214</v>
       </c>
       <c r="B89" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C89">
-        <v>261581</v>
+        <v>435351</v>
       </c>
       <c r="D89" t="s">
         <v>215</v>
@@ -2445,10 +2481,10 @@
         <v>216</v>
       </c>
       <c r="B90" t="s">
-        <v>69</v>
+        <v>52</v>
       </c>
       <c r="C90">
-        <v>444705</v>
+        <v>1107516</v>
       </c>
       <c r="D90" t="s">
         <v>217</v>
@@ -2459,10 +2495,10 @@
         <v>218</v>
       </c>
       <c r="B91" t="s">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="C91">
-        <v>1054569</v>
+        <v>612392</v>
       </c>
       <c r="D91" t="s">
         <v>219</v>
@@ -2473,10 +2509,10 @@
         <v>220</v>
       </c>
       <c r="B92" t="s">
-        <v>69</v>
+        <v>5</v>
       </c>
       <c r="C92">
-        <v>435351</v>
+        <v>672992</v>
       </c>
       <c r="D92" t="s">
         <v>221</v>
@@ -2487,10 +2523,10 @@
         <v>222</v>
       </c>
       <c r="B93" t="s">
-        <v>54</v>
+        <v>109</v>
       </c>
       <c r="C93">
-        <v>1107516</v>
+        <v>1541013</v>
       </c>
       <c r="D93" t="s">
         <v>223</v>
@@ -2501,94 +2537,94 @@
         <v>224</v>
       </c>
       <c r="B94" t="s">
-        <v>8</v>
+        <v>225</v>
       </c>
       <c r="C94">
-        <v>612392</v>
+        <v>34512</v>
       </c>
       <c r="D94" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B95" t="s">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="C95">
-        <v>672992</v>
+        <v>1015999</v>
       </c>
       <c r="D95" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B96" t="s">
-        <v>113</v>
+        <v>52</v>
       </c>
       <c r="C96">
-        <v>1541013</v>
+        <v>1111957</v>
       </c>
       <c r="D96" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B97" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C97">
-        <v>34512</v>
+        <v>24665</v>
       </c>
       <c r="D97" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B98" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C98">
-        <v>1015999</v>
+        <v>1212312</v>
       </c>
       <c r="D98" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B99" t="s">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="C99">
-        <v>1111957</v>
+        <v>1020051</v>
       </c>
       <c r="D99" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B100" t="s">
-        <v>238</v>
+        <v>34</v>
       </c>
       <c r="C100">
-        <v>24665</v>
+        <v>1287248</v>
       </c>
       <c r="D100" t="s">
         <v>239</v>
@@ -2598,13 +2634,13 @@
       <c r="A101" t="s">
         <v>240</v>
       </c>
-      <c r="B101">
-        <v>2023</v>
+      <c r="B101" t="s">
+        <v>85</v>
       </c>
       <c r="C101">
-        <v>1212312</v>
-      </c>
-      <c r="D101" s="2" t="s">
+        <v>52252</v>
+      </c>
+      <c r="D101" t="s">
         <v>241</v>
       </c>
     </row>
@@ -2612,13 +2648,13 @@
       <c r="A102" t="s">
         <v>242</v>
       </c>
-      <c r="B102">
-        <v>2022</v>
+      <c r="B102" t="s">
+        <v>85</v>
       </c>
       <c r="C102">
-        <v>1020051</v>
-      </c>
-      <c r="D102" s="2" t="s">
+        <v>47911</v>
+      </c>
+      <c r="D102" t="s">
         <v>243</v>
       </c>
     </row>
@@ -2626,160 +2662,229 @@
       <c r="A103" t="s">
         <v>244</v>
       </c>
-      <c r="B103">
-        <v>2024</v>
+      <c r="B103" t="s">
+        <v>245</v>
       </c>
       <c r="C103">
-        <v>1287248</v>
+        <v>26621</v>
       </c>
       <c r="D103" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
-        <v>246</v>
-      </c>
-      <c r="B104">
-        <v>2010</v>
+        <v>247</v>
+      </c>
+      <c r="B104" t="s">
+        <v>14</v>
       </c>
       <c r="C104">
-        <v>52252</v>
+        <v>110549</v>
       </c>
       <c r="D104" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
-        <v>248</v>
-      </c>
-      <c r="B105">
-        <v>2010</v>
+        <v>249</v>
+      </c>
+      <c r="B105" t="s">
+        <v>64</v>
       </c>
       <c r="C105">
-        <v>47911</v>
+        <v>456193</v>
       </c>
       <c r="D105" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
-        <v>250</v>
-      </c>
-      <c r="B106">
-        <v>2009</v>
+        <v>251</v>
+      </c>
+      <c r="B106" t="s">
+        <v>23</v>
       </c>
       <c r="C106">
-        <v>26621</v>
+        <v>937348</v>
       </c>
       <c r="D106" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
-        <v>252</v>
-      </c>
-      <c r="B107">
-        <v>2012</v>
+        <v>253</v>
+      </c>
+      <c r="B107" t="s">
+        <v>64</v>
       </c>
       <c r="C107">
-        <v>110549</v>
+        <v>484413</v>
       </c>
       <c r="D107" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
-        <v>254</v>
-      </c>
-      <c r="B108">
-        <v>2017</v>
+        <v>255</v>
+      </c>
+      <c r="B108" t="s">
+        <v>256</v>
       </c>
       <c r="C108">
-        <v>456193</v>
+        <v>198306</v>
       </c>
       <c r="D108" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
-        <v>256</v>
-      </c>
-      <c r="B109">
-        <v>2022</v>
+        <v>258</v>
+      </c>
+      <c r="B109" t="s">
+        <v>64</v>
       </c>
       <c r="C109">
-        <v>937348</v>
+        <v>442087</v>
       </c>
       <c r="D109" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
-        <v>258</v>
-      </c>
-      <c r="B110">
-        <v>2017</v>
+        <v>260</v>
+      </c>
+      <c r="B110" t="s">
+        <v>14</v>
       </c>
       <c r="C110">
-        <v>484413</v>
+        <v>84154</v>
       </c>
       <c r="D110" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
-        <v>260</v>
-      </c>
-      <c r="B111">
-        <v>2003</v>
+        <v>262</v>
+      </c>
+      <c r="B111" t="s">
+        <v>109</v>
       </c>
       <c r="C111">
-        <v>198306</v>
+        <v>1442369</v>
       </c>
       <c r="D111" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
-        <v>262</v>
-      </c>
-      <c r="B112">
-        <v>2017</v>
+        <v>264</v>
+      </c>
+      <c r="B112" t="s">
+        <v>57</v>
       </c>
       <c r="C112">
-        <v>442087</v>
+        <v>26775</v>
       </c>
       <c r="D112" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
-        <v>264</v>
-      </c>
-      <c r="B113">
-        <v>2012</v>
+        <v>266</v>
+      </c>
+      <c r="B113" t="s">
+        <v>26</v>
       </c>
       <c r="C113">
-        <v>84154</v>
+        <v>419219</v>
       </c>
       <c r="D113" t="s">
-        <v>265</v>
+        <v>267</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A114" t="s">
+        <v>268</v>
+      </c>
+      <c r="B114" t="s">
+        <v>29</v>
+      </c>
+      <c r="C114">
+        <v>573443</v>
+      </c>
+      <c r="D114" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A115" t="s">
+        <v>270</v>
+      </c>
+      <c r="B115" t="s">
+        <v>75</v>
+      </c>
+      <c r="C115">
+        <v>52153</v>
+      </c>
+      <c r="D115" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A116" t="s">
+        <v>272</v>
+      </c>
+      <c r="B116" t="s">
+        <v>34</v>
+      </c>
+      <c r="C116">
+        <v>1247759</v>
+      </c>
+      <c r="D116" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A117" t="s">
+        <v>274</v>
+      </c>
+      <c r="B117">
+        <v>1987</v>
+      </c>
+      <c r="C117">
+        <v>17159</v>
+      </c>
+      <c r="D117" s="2" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A118" t="s">
+        <v>276</v>
+      </c>
+      <c r="B118">
+        <v>2021</v>
+      </c>
+      <c r="C118">
+        <v>823754</v>
+      </c>
+      <c r="D118" t="s">
+        <v>277</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D101" r:id="rId1" xr:uid="{419420B0-79EB-44E4-B02A-6B12850B061F}"/>
-    <hyperlink ref="D102" r:id="rId2" xr:uid="{7B2A5A40-BC38-4883-8EB3-BC0C9A5C6138}"/>
+    <hyperlink ref="D117" r:id="rId1" xr:uid="{6B9312CA-D6D6-4D45-A664-3A66B9736370}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adding batching for whitelist updates
</commit_message>
<xml_diff>
--- a/Comedy_Whitelist.xlsx
+++ b/Comedy_Whitelist.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bigba\aa Personal Projects\Letterboxd-List-Scraping\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B42148C-FAA6-4007-93DA-CBC3DD5FE732}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D8BADF8-3C14-47F3-850A-FC19561BC553}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2080" yWindow="2080" windowWidth="14400" windowHeight="8170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="280">
   <si>
     <t>Title</t>
   </si>
@@ -854,6 +854,12 @@
   </si>
   <si>
     <t>https://letterboxd.com/film/bo-burnham-inside/</t>
+  </si>
+  <si>
+    <t>Stewart Lee: Content Provider</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/stewart-lee-content-provider/</t>
   </si>
 </sst>
 </file>
@@ -1227,7 +1233,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D118"/>
+  <dimension ref="A1:D119"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
@@ -2880,6 +2886,20 @@
       </c>
       <c r="D118" t="s">
         <v>277</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A119" t="s">
+        <v>278</v>
+      </c>
+      <c r="B119">
+        <v>2018</v>
+      </c>
+      <c r="C119">
+        <v>530349</v>
+      </c>
+      <c r="D119" t="s">
+        <v>279</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Making less memory consuming
</commit_message>
<xml_diff>
--- a/Comedy_Whitelist.xlsx
+++ b/Comedy_Whitelist.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bigba\aa Personal Projects\Letterboxd-List-Scraping\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D6A3F53-AACD-4CF9-93DB-DBCAE15D3327}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5B4AC4A-A1B6-4FC4-959E-C08F45D18E01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="287">
   <si>
     <t>Title</t>
   </si>
@@ -866,6 +866,21 @@
   </si>
   <si>
     <t>https://letterboxd.com/film/deniz-goktas-olu-deniz/</t>
+  </si>
+  <si>
+    <t>Chris Fleming: Showpig</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/chris-fleming-showpig/</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/daniel-sloss-socio/</t>
+  </si>
+  <si>
+    <t>Daniel Sloss: Socio</t>
   </si>
 </sst>
 </file>
@@ -1239,7 +1254,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D120"/>
+  <dimension ref="A1:E122"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
@@ -2810,7 +2825,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>266</v>
       </c>
@@ -2824,7 +2839,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>268</v>
       </c>
@@ -2838,7 +2853,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>270</v>
       </c>
@@ -2852,7 +2867,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>272</v>
       </c>
@@ -2866,7 +2881,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>274</v>
       </c>
@@ -2880,7 +2895,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>276</v>
       </c>
@@ -2894,7 +2909,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>278</v>
       </c>
@@ -2908,7 +2923,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>280</v>
       </c>
@@ -2920,12 +2935,44 @@
       </c>
       <c r="D120" s="2" t="s">
         <v>281</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A121" t="s">
+        <v>282</v>
+      </c>
+      <c r="B121">
+        <v>2018</v>
+      </c>
+      <c r="C121">
+        <v>526530</v>
+      </c>
+      <c r="D121" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A122" t="s">
+        <v>286</v>
+      </c>
+      <c r="B122">
+        <v>2022</v>
+      </c>
+      <c r="C122">
+        <v>1054105</v>
+      </c>
+      <c r="D122" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="E122" t="s">
+        <v>284</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D117" r:id="rId1" xr:uid="{6B9312CA-D6D6-4D45-A664-3A66B9736370}"/>
     <hyperlink ref="D120" r:id="rId2" xr:uid="{B5127FF8-3570-49A7-91BC-B126EB18D554}"/>
+    <hyperlink ref="D122" r:id="rId3" xr:uid="{47150D12-8DC3-428F-AB07-31014E62FB05}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>